<commit_message>
Chỉnh sửa preprocessing + checking plots
</commit_message>
<xml_diff>
--- a/results/data_quality_report/clip_summary.xlsx
+++ b/results/data_quality_report/clip_summary.xlsx
@@ -467,19 +467,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="C2" t="n">
-        <v>-46800</v>
+        <v>-21750</v>
       </c>
       <c r="D2" t="n">
-        <v>70100</v>
+        <v>45050</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>4577</v>
+        <v>6404</v>
       </c>
     </row>
     <row r="3">

</xml_diff>